<commit_message>
/start landing: product page handoff, OTTO cap
</commit_message>
<xml_diff>
--- a/custom-products.xlsx
+++ b/custom-products.xlsx
@@ -675,17 +675,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>LOCAL-001</t>
+          <t>31-069</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Local Supplier Trucker Hat</t>
+          <t>OTTO CAP 5 Panel Mid Profile Baseball Cap</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Local Supplier</t>
+          <t>OTTO CAP</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -695,25 +695,23 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Trucker Hat</t>
+          <t>Baseball Caps</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Foam-front, mesh-back, snapback.</t>
+          <t>65/35 polyester/cotton twill. Structured firm front panel. Mid profile. Pre-curved visor. Adjustable snapback. One size fits most.</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>6.5</v>
+        <v>5.05</v>
       </c>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n">
-        <v>12</v>
-      </c>
+      <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
@@ -725,88 +723,34 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>OS</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr"/>
+          <t>OSFA</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>[{"name":"Black","code":"BK","hex":"#000000","images":{"front_model":"https://example.com/local-001-black-front.jpg","back_model":"https://example.com/local-001-black-back.jpg","front_flat":null,"back_flat":null,"side_model":null}},{"name":"White","code":"WH","hex":"#FFFFFF","images":{"front_model":"https://example.com/local-001-white-front.jpg","back_model":null,"front_flat":null,"back_flat":null,"side_model":null}}]</t>
+          <t>[{"name": "Black", "code": "003", "hex": "#000000", "images": {"front_model": "https://aliveprintshop.github.io/PriceCalculator/media/otto-31069-black-front.jpg", "back_model": "https://aliveprintshop.github.io/PriceCalculator/media/otto-31069-black-back.jpg", "front_flat": "https://aliveprintshop.github.io/PriceCalculator/media/otto-31069-black-front.jpg", "back_flat": "https://aliveprintshop.github.io/PriceCalculator/media/otto-31069-black-back.jpg", "side_model": null}}]</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>LOCAL-002</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Seasonal Clearance Tote</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Local Supplier</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Tote</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Canvas tote, 12oz. Limited time pricing.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>4.95</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Regular</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>OS</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>[{"name":"Navy","code":"NVY","hex":"#1B2C55","images":{"front_model":"https://example.com/local-002-navy-front.jpg","back_model":null,"front_flat":null,"back_flat":null,"side_model":null}}]</t>
-        </is>
-      </c>
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>